<commit_message>
Word documents v1.1 for the Habmann feedback: trainer documents, lesson plan, AI notice, Document use sheet
- Add a Trainer document per day (Day 1-8): coaching UE4, case-study and transfer model solutions, feedback round, assessment criteria, transition from Level 2 to 3
- Add "Day at a glance" (UE1-UE10) to every document; mark case study 2 UE (UE5-6) and transfer project 3 UE (UE8-10); UE column in the Task coverage tables
- Add AI notice (EN/DE), version 1.1, release date 14.10.2026 and named approver to every cover and footer; label every figure with "AI" on the image
- Add block orientation to the Day 1 Materi, a "Use in class: presentation and handout" table and the playground addresses to every document
- Add the sheet "Document use Day 1-8" to the One Stop plan workbook
- CLAUDE.md #53 (Word-only rules); correct #50: the plan merges UE8-10 into the transfer project

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/One Stop Digital Learning - Strukturplan 11_F_128 (04-26).xlsx
+++ b/One Stop Digital Learning - Strukturplan 11_F_128 (04-26).xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deutsch" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bahasa Indonesia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document use Day 1-8" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -193,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -260,6 +261,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -4505,76 +4509,31 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="C31" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39">
       <c r="C39" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
     <row r="47">
       <c r="C47" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="C56" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
     <row r="65">
       <c r="C65" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
     <row r="75">
       <c r="C75" t="n">
         <v>8</v>
@@ -7481,76 +7440,31 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="C31" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39">
       <c r="C39" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
     <row r="47">
       <c r="C47" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="C56" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
     <row r="65">
       <c r="C65" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
     <row r="75">
       <c r="C75" t="n">
         <v>8</v>
@@ -10457,76 +10371,31 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="C31" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39">
       <c r="C39" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
     <row r="47">
       <c r="C47" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="C56" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
     <row r="65">
       <c r="C65" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
     <row r="75">
       <c r="C75" t="n">
         <v>8</v>
@@ -10576,4 +10445,1057 @@
   <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001750A8"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UE</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Methodology</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 3</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 4</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 5</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 6</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 7</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Documents - Day 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="81" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Topic of the Day</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Module 1 (Day 1 of 2) Fundamentals of UX/UI Design for Digital Learning Platforms &amp; User-Centered Design of Learning Interfaces</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Module 1 (Day 2 of 2) Practical Analysis of Successful E-Learning Platforms, Prototyping &amp; Testing of Learning Interfaces, Future Technologies &amp; Adaptive Learning Systems</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Module 2 (Day 1 of 2): Fundamentals of Learning Psychology for UX Designers &amp; Cognitive Load and Information Processing</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Module 2 (Day 2 of 2): Motivation and Engagement through Design Psychology, Design Principles for Effective Learning Experiences, Evaluation and Optimization of Learning-Psychology-Based UX Concepts</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Module 3 (Day 1 of 3): Fundamentals of User-Centered UX Design for Learning Platforms</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Module 3 (Day 2 of 3): Developing Personas for Learners and Teachers &amp; Mapping User Journeys in the Learning Context</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Module 3 (Day 3 of 3): Accessibility and Inclusive Design of Learning Platforms &amp; Integration and Evaluation of User-Centered UX Concepts</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Module 4 (Day 1 of 3): Fundamentals of UX/UI Design for Digital Learning Environments</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="141" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Documents (version 1.1)</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day1-Materi-Habmann-Digital-Learning-UX-vs-UI-and-User-Centred-Design.docx
+Task: Day1-Task-Habmann-Digital-Learning-LearnFast-UX-Analysis-and-UX-Strategy-Memo.docx
+Trainer (not for participants): Day1-Trainer-Habmann-Digital-Learning-SkillUp-and-LearnFast-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day2-Materi-Habmann-Digital-Learning-Successful-Platforms-Prototyping-Testing-and-Adaptive-Learning.docx
+Task: Day2-Task-Habmann-Digital-Learning-LearnPro-Prototype-and-Test-Plan-and-Innovation-Strategy.docx
+Trainer (not for participants): Day2-Trainer-Habmann-Digital-Learning-LearnPro-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day3-Materi-Habmann-Digital-Learning-Learning-Psychology-and-Cognitive-Load.docx
+Task: Day3-Task-Habmann-Digital-Learning-EduCore-Cognitive-Load-Analysis-and-Learning-Experience-Strategy.docx
+Trainer (not for participants): Day3-Trainer-Habmann-Digital-Learning-EduCore-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day4-Materi-Habmann-Digital-Learning-Motivation-and-Engagement-by-Design.docx
+Task: Day4-Task-Habmann-Digital-Learning-MotivaLearn-Engagement-Analysis-and-Engagement-Strategy.docx
+Trainer (not for participants): Day4-Trainer-Habmann-Digital-Learning-MotivaLearn-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day5-Materi-Habmann-Digital-Learning-User-Centred-UX-Design.docx
+Task: Day5-Task-Habmann-Digital-Learning-LearnBase-User-Centred-Analysis-and-UX-Strategy.docx
+Trainer (not for participants): Day5-Trainer-Habmann-Digital-Learning-LearnBase-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day6-Materi-Habmann-Digital-Learning-Personas-and-User-Journeys.docx
+Task: Day6-Task-Habmann-Digital-Learning-EduPath-Personas-Journeys-and-Segmentation-Strategy.docx
+Trainer (not for participants): Day6-Trainer-Habmann-Digital-Learning-EduPath-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day7-Materi-Habmann-Digital-Learning-Accessibility-and-Inclusive-Design.docx
+Task: Day7-Task-Habmann-Digital-Learning-InclusiveLearn-Barrier-Analysis-and-Inclusive-UX-Strategy.docx
+Trainer (not for participants): Day7-Trainer-Habmann-Digital-Learning-InclusiveLearn-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Materi: Day8-Materi-Habmann-Digital-Learning-UX-UI-Structure-Visual-Hierarchy-and-Interaction.docx
+Task: Day8-Task-Habmann-Digital-Learning-StructLearn-Structure-Analysis-and-Basic-UX-UI-Structure.docx
+Trainer (not for participants): Day8-Trainer-Habmann-Digital-Learning-StructLearn-Coaching-Feedback-and-Model-Solutions.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="66" customHeight="1">
+      <c r="A4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Level 1 Knowledge</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Knowledge Transfer</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 50 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 50 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 50 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 50 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 48 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 50 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 48 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>MATERI A (Route 1)
+Core cards A1, A2, A3, A5 (about 50 min).
+Optional A4: handout only.
+Format: Presentation + Handout</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="51" customHeight="1">
+      <c r="A5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Level 1 Task 1</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Structuring Fundamentals</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.1 (Core, about 13 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
+      <c r="A6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Level 1 Task 2</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Evaluation and Prioritization</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 2
+Block 2.2 (Core, about 17 min): rating part; finished in UE5–6.
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>TASK 1 · Part 1
+Block 1.2 (Optional, about 8 min).
+Format: Handout (or on the playground)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Level 1 + 2 Coaching</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Coaching Topics: Transition into Application</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>COACHING
+TASK 1 · Block 1.3 (Optional, about 5 min).
+TRAINER document, section Coaching.
+Format: Trainer only + Handout</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Level 2 Application (Case study, 2 UE)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Case Study (2 UE) incl. Model Solution</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY SkillUp · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY LearnPro · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY EduCore · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY MotivaLearn · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY LearnBase · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY EduPath · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY InclusiveLearn · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>CASE STUDY StructLearn · 2 UE
+TASK 1 · Part 2: Block 2.1 (Optional, about 7 min); Block 2.2 (Core, about 17 min).
+UE5: brief and own work. UE6: groups compare; the model solution is shown at the end (TRAINER document, section Case study).
+Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="81" customHeight="1">
+      <c r="A10" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Level 2 + 3 Feedback</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Feedback Round with a Management Perspective</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>FEEDBACK ROUND
+TRAINER document, section Feedback round (groups present their reasoning; Level 3 input questions).
+Format: Presentation by the groups; Trainer only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52.66666666666666" customHeight="1">
+      <c r="A11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Senior Level 3 Transfer Project (3 UE)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Project Work – Developing Decision Architecture</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief UX Officer · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief Product Officer · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief Learning Experience Officer · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief Experience Officer · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief UX Strategist · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Head of UX Strategy · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief UX &amp; Accessibility Officer · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 9 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 11 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>TRANSFER PROJECT · Chief UX Architect · 3 UE
+UE8: MATERI B, Core cards B1, B2, B3. Format: Presentation + Handout.
+UE9: TASK 2, Block 3.1 (Core, about 10 min). Format: Handout.
+UE10: TASK 2, Block 3.2 (Core, about 10 min); then debrief with the model solution (TRAINER document, section Transfer project). Format: Handout; model solution shown after the work</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52.66666666666666" customHeight="1">
+      <c r="A12" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="25" t="n"/>
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="52.66666666666666" customHeight="1">
+      <c r="A13" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Playground (website)</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/1/</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/2/</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/3/</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/4/</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/5/</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/6/</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/7/</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>https://aion-dl.vercel.app/day/8/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Version, date, approval</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Version 1.1 · 14.10.2026
+Review and approval: Muhammad Muchson, Mentor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>How to read this sheet</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n"/>
+      <c r="C17" s="1" t="n"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>MATERI</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>The study material of the day. Materi A serves Route 1 (Levels 1 and 2), Materi B serves Route 2 (Level 3). Participants get it as a handout; the trainer presents the Core cards on the playground.</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>TASK</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>The worksheet of the day. Task 1 is Route 1 (Part 1 = Level 1, Part 2 = the Level 2 case study, 2 UE). Task 2 is Route 2, the Level 3 transfer project (3 UE). It carries no answer keys and no scores. Participants get it as a handout or work in it on the playground.</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Coaching, feedback round, model solutions (Musterlösung), assessment criteria (Bewertungskriterien) and the transition from Level 2 to Level 3. Not handed out to participants. Model solutions are shown only after the participants have worked.</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Presentation / Handout</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Presentation = what the trainer shows on screen (the cards' scan line, figures and key boxes; the case; the model solution after the work). Handout = what participants read, fill in and keep.</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>PLAYGROUND</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>The course website (https://aion-dl.vercel.app/): in class it is the place to practise and learn. Each day has its own address: https://aion-dl.vercel.app/day/N/.</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>UE</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>One teaching unit (Unterrichtseinheit) is counted as 45 minutes; breaks are not shown. The case study is 2 UE (UE5–6), the transfer project 3 UE (UE8–10).</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="37">
+    <mergeCell ref="D20:K20"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="D19:K19"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="E11:E13"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D22:K22"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D21:K21"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="F11:F13"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="G11:G13"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="I11:I13"/>
+    <mergeCell ref="K11:K13"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D18:K18"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="J11:J13"/>
+    <mergeCell ref="D23:K23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>